<commit_message>
Create README for scripts
</commit_message>
<xml_diff>
--- a/data/raw/Treatment_Info_columns.xlsx
+++ b/data/raw/Treatment_Info_columns.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eltnmsu-my.sharepoint.com/personal/lossanna_nmsu_edu/Documents/Documents/04_LDC-LTDL/LDC-LTDL/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="294" documentId="8_{48365B36-8811-40C8-A04C-04A62785130B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8BD2CCD5-C082-4C12-A71E-4DCF7E2A6EF8}"/>
+  <xr:revisionPtr revIDLastSave="299" documentId="8_{48365B36-8811-40C8-A04C-04A62785130B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7D749C2E-E32A-4DD3-B580-6E806271167A}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="1620" windowWidth="20376" windowHeight="12096" activeTab="1" xr2:uid="{180FE257-6980-4323-B5A2-AB4BD0017CAE}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="80">
   <si>
     <t>Column</t>
   </si>
@@ -271,6 +271,12 @@
   </si>
   <si>
     <t>If the treatment included seeding ("-1" means seeding occurred)</t>
+  </si>
+  <si>
+    <t>6 options</t>
+  </si>
+  <si>
+    <t>Status of the seed list (confirmed/unknown/planned, etc.)</t>
   </si>
 </sst>
 </file>
@@ -919,6 +925,15 @@
       <c r="A15" t="s">
         <v>34</v>
       </c>
+      <c r="B15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">

</xml_diff>

<commit_message>
Create README for LTDL-versions folder
</commit_message>
<xml_diff>
--- a/data/raw/Treatment_Info_columns.xlsx
+++ b/data/raw/Treatment_Info_columns.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eltnmsu-my.sharepoint.com/personal/lossanna_nmsu_edu/Documents/Documents/04_LDC-LTDL/LDC-LTDL/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="299" documentId="8_{48365B36-8811-40C8-A04C-04A62785130B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7D749C2E-E32A-4DD3-B580-6E806271167A}"/>
+  <xr:revisionPtr revIDLastSave="301" documentId="8_{48365B36-8811-40C8-A04C-04A62785130B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{10B9F0AF-BCF8-4F80-B629-0183F98E2FCF}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="1620" windowWidth="20376" windowHeight="12096" activeTab="1" xr2:uid="{180FE257-6980-4323-B5A2-AB4BD0017CAE}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="80">
   <si>
     <t>Column</t>
   </si>
@@ -687,7 +687,7 @@
         <v>9</v>
       </c>
       <c r="B2" s="2">
-        <v>45994</v>
+        <v>45995</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
@@ -940,82 +940,85 @@
         <v>35</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="B26" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>47</v>
       </c>

</xml_diff>

<commit_message>
Continue working on treatment info
</commit_message>
<xml_diff>
--- a/data/raw/Treatment_Info_columns.xlsx
+++ b/data/raw/Treatment_Info_columns.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eltnmsu-my.sharepoint.com/personal/lossanna_nmsu_edu/Documents/Documents/04_LDC-LTDL/LDC-LTDL/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="301" documentId="8_{48365B36-8811-40C8-A04C-04A62785130B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{10B9F0AF-BCF8-4F80-B629-0183F98E2FCF}"/>
+  <xr:revisionPtr revIDLastSave="355" documentId="8_{48365B36-8811-40C8-A04C-04A62785130B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A779CA46-2FFC-4213-A19F-A46BE165530F}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="1620" windowWidth="20376" windowHeight="12096" activeTab="1" xr2:uid="{180FE257-6980-4323-B5A2-AB4BD0017CAE}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="113">
   <si>
     <t>Column</t>
   </si>
@@ -277,6 +277,105 @@
   </si>
   <si>
     <t>Status of the seed list (confirmed/unknown/planned, etc.)</t>
+  </si>
+  <si>
+    <t>Point; Polygon; Polyline; Multipoint</t>
+  </si>
+  <si>
+    <t>GIS feature geometry</t>
+  </si>
+  <si>
+    <t>Name of seed mix (possibly connects to Seed_Species.csv</t>
+  </si>
+  <si>
+    <t>Seeds; Seedlings; Unknown; NA</t>
+  </si>
+  <si>
+    <t>If seeds or seedlings were planted</t>
+  </si>
+  <si>
+    <t>8 options</t>
+  </si>
+  <si>
+    <t>If seed list was confirmed (confirmed/unknown/planned, etc.)</t>
+  </si>
+  <si>
+    <t>7 options</t>
+  </si>
+  <si>
+    <t>If a control area was established</t>
+  </si>
+  <si>
+    <t>Species Specific; Overall; Unknown; Not Available; NA</t>
+  </si>
+  <si>
+    <t>Honestly idk</t>
+  </si>
+  <si>
+    <t>Additional notes about seeding</t>
+  </si>
+  <si>
+    <t>List of objectives (level of description varies)</t>
+  </si>
+  <si>
+    <t>Planned implementation</t>
+  </si>
+  <si>
+    <t>Actual implementation</t>
+  </si>
+  <si>
+    <t>Treatment effect and results</t>
+  </si>
+  <si>
+    <t>Approximate point; Confirmed; Planned; Unknown; confirmed</t>
+  </si>
+  <si>
+    <t>If the feature location is confirmed</t>
+  </si>
+  <si>
+    <t>How the feature was created (usually some kind of digitization)</t>
+  </si>
+  <si>
+    <t>22 options</t>
+  </si>
+  <si>
+    <t>Number of acres</t>
+  </si>
+  <si>
+    <t>This can differ from the GIS geometry shape area because it was what was measured on the ground (e.g., sometimes there's a big rock pile and that isn't counted)</t>
+  </si>
+  <si>
+    <t>The number of acres on BLM land (I think?)</t>
+  </si>
+  <si>
+    <t>Notes about GIS</t>
+  </si>
+  <si>
+    <t>Who initiated the project (BLM/contractor, etc.)</t>
+  </si>
+  <si>
+    <t>9 options</t>
+  </si>
+  <si>
+    <t>Concerns about treatment</t>
+  </si>
+  <si>
+    <t>Notes about treatment</t>
+  </si>
+  <si>
+    <t>Description of treatment concerns</t>
+  </si>
+  <si>
+    <t>Problems when applying treatment</t>
+  </si>
+  <si>
+    <t>Description of problems when applying treatment</t>
+  </si>
+  <si>
+    <t>Conditions at time of treatment</t>
+  </si>
+  <si>
+    <t>Description about conditions at time of treatment</t>
   </si>
 </sst>
 </file>
@@ -939,128 +1038,305 @@
       <c r="A16" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B16" t="s">
+        <v>74</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B17" t="s">
+        <v>59</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B18" t="s">
+        <v>59</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B19" t="s">
+        <v>59</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B20" t="s">
+        <v>59</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B21" t="s">
+        <v>74</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B22" t="s">
+        <v>74</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B23" t="s">
+        <v>74</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B24" t="s">
+        <v>74</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B25" t="s">
+        <v>74</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>45</v>
       </c>
       <c r="B26" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="C26" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B27" t="s">
+        <v>59</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B28" t="s">
+        <v>59</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B29" t="s">
+        <v>65</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B30" t="s">
+        <v>6</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B31" t="s">
+        <v>6</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>47</v>
+      </c>
+      <c r="B32" t="s">
+        <v>74</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>48</v>
       </c>
+      <c r="B33" t="s">
+        <v>59</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="E33" s="4" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>49</v>
       </c>
+      <c r="B34" t="s">
+        <v>74</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>106</v>
+      </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>50</v>
       </c>
+      <c r="B35" t="s">
+        <v>74</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>108</v>
+      </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>51</v>
       </c>
+      <c r="B36" t="s">
+        <v>74</v>
+      </c>
+      <c r="D36" s="4" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>52</v>
       </c>
+      <c r="B37" t="s">
+        <v>74</v>
+      </c>
+      <c r="D37" s="4" t="s">
+        <v>110</v>
+      </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>53</v>
       </c>
+      <c r="B38" t="s">
+        <v>74</v>
+      </c>
+      <c r="D38" s="4" t="s">
+        <v>111</v>
+      </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>54</v>
       </c>
+      <c r="B39" t="s">
+        <v>74</v>
+      </c>
+      <c r="D39" s="4" t="s">
+        <v>112</v>
+      </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>55</v>
+      </c>
+      <c r="B40" t="s">
+        <v>74</v>
+      </c>
+      <c r="D40" s="4" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="41" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">

</xml_diff>